<commit_message>
lab2 - docs testlink
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="5"/>
+  <fileVersion appName="Calc" lowestEdited="7"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="89">
   <si>
     <t xml:space="preserve">do not print this form</t>
   </si>
@@ -163,12 +163,6 @@
     <t xml:space="preserve">Stoc contine cantitate si stoc minim de tip double dar in constructor apare ca int</t>
   </si>
   <si>
-    <t xml:space="preserve">A03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tip si categoria sunt trecute ca enum, dar in cerinta exista o functionalitate ce ii permite userului sa adauge tipuri si categori</t>
-  </si>
-  <si>
     <t xml:space="preserve">A05</t>
   </si>
   <si>
@@ -184,6 +178,30 @@
     <t xml:space="preserve">Popescu Ionel</t>
   </si>
   <si>
+    <t xml:space="preserve">05.03.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comenzile au nevoie de un atribut LocalDateTime, pentru a putea crea raportul zilnic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nu este afisat in ui stockul ingredientelor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nu tine cont de stock cand faci o comanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In constructorul Stoc cantitate si stocMinim apare ca int, dar tipul variabilelor este double</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tool-based Code Analysis</t>
   </si>
   <si>
@@ -202,7 +220,76 @@
     <t xml:space="preserve">After/Argument</t>
   </si>
   <si>
-    <t xml:space="preserve">Effort to perform tool-based code analysis (hours):</t>
+    <t xml:space="preserve">AbstractRepository,37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methods should not have identical implementations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metodele sunt păstrate separat pentru a reflecta operațiile CRUD, chiar daca implementarea actuală este identică</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CsvExporter,14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utility classes should not have public constructors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nu era definit un constructor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Am definit un constructor privat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AbstractRepository,20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redundant casts should not be used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se făcea cast la List&lt;E&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Am șters cast-ul redundant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FileAbstractRepository,12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constructors of an "abstract" class should not be declared "public"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constructorul era declarat public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constructorul e declarat protected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FileOrderRepository, 59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">String.isEmpty() should be used to test for emptiness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se verifica dacă stringbuilder-ul e gol folosind .lenght()&gt;0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se foloseste .isEmpty() pentru a verifica dacă stringbuilder-ul este gol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CsvExporter,11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unnecessary imports should be removed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se importa ceva ce nu era folosit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S-a șters importul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effort to perform tool-based code analysis (hours): 0.3</t>
   </si>
 </sst>
 </file>
@@ -212,7 +299,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,13 +376,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <charset val="238"/>
     </font>
   </fonts>
@@ -308,19 +388,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999"/>
+        <fgColor theme="7" tint="0.7998"/>
         <bgColor rgb="FFEBF1DE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999"/>
+        <fgColor theme="9" tint="0.7998"/>
         <bgColor rgb="FFEBF1DE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.7999"/>
+        <fgColor theme="3" tint="0.7998"/>
         <bgColor rgb="FFE6E0EC"/>
       </patternFill>
     </fill>
@@ -387,7 +467,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -452,10 +532,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -484,7 +560,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -498,6 +574,18 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -762,17 +850,17 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.91015625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="29.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.45"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.91"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="29.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.45"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="1" width="8.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.42"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="1" width="8.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -786,7 +874,7 @@
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
@@ -801,7 +889,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
@@ -812,7 +900,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C4" s="7" t="s">
         <v>7</v>
       </c>
@@ -830,7 +918,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="7" t="s">
         <v>11</v>
       </c>
@@ -848,7 +936,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="10"/>
       <c r="C6" s="11" t="s">
         <v>15</v>
@@ -856,7 +944,7 @@
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="11" t="s">
         <v>16</v>
       </c>
@@ -865,7 +953,7 @@
       </c>
       <c r="E7" s="12"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13" t="s">
         <v>18</v>
       </c>
@@ -886,10 +974,10 @@
       <c r="C10" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="16" t="s">
         <v>24</v>
       </c>
     </row>
@@ -904,7 +992,7 @@
       <c r="D11" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>26</v>
       </c>
     </row>
@@ -917,7 +1005,7 @@
         <v>27</v>
       </c>
       <c r="D12" s="15"/>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="16" t="s">
         <v>28</v>
       </c>
     </row>
@@ -932,11 +1020,11 @@
       <c r="D13" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="16" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="n">
         <f aca="false">B13+1</f>
         <v>5</v>
@@ -945,7 +1033,7 @@
         <v>27</v>
       </c>
       <c r="D14" s="15"/>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="16" t="s">
         <v>30</v>
       </c>
     </row>
@@ -960,11 +1048,11 @@
       <c r="D15" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
@@ -975,96 +1063,96 @@
       <c r="D16" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
-      <c r="E17" s="17"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E17" s="16"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="n">
         <f aca="false">B17+1</f>
         <v>9</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
-      <c r="E18" s="18"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E18" s="17"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="n">
         <f aca="false">B18+1</f>
         <v>10</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="18"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E19" s="17"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="n">
         <f aca="false">B19+1</f>
         <v>11</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="18"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E20" s="17"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="n">
         <f aca="false">B20+1</f>
         <v>12</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
-      <c r="E21" s="18"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E21" s="17"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="n">
         <f aca="false">B21+1</f>
         <v>13</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
-      <c r="E22" s="18"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E22" s="17"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="n">
         <f aca="false">B22+1</f>
         <v>14</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
-      <c r="E23" s="18"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E23" s="17"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="n">
         <f aca="false">B23+1</f>
         <v>15</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
-      <c r="E24" s="18"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E24" s="17"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="n">
         <f aca="false">B24+1</f>
         <v>16</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
-      <c r="E25" s="18"/>
-    </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="19" t="s">
+      <c r="E25" s="17"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C27" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="20"/>
+      <c r="D27" s="19"/>
       <c r="E27" s="15" t="n">
         <v>0.5</v>
       </c>
@@ -1095,15 +1183,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.91015625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="16.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.45"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.09"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.91"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="16.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1117,7 +1205,7 @@
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
         <v>37</v>
       </c>
@@ -1132,7 +1220,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
@@ -1143,14 +1231,14 @@
         <v>233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="21" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C4" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="22"/>
+      <c r="E4" s="21"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1161,14 +1249,14 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="21" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="23"/>
+      <c r="E5" s="22"/>
       <c r="H5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1179,7 +1267,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="10"/>
       <c r="C6" s="11" t="s">
         <v>15</v>
@@ -1187,14 +1275,16 @@
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="12" t="s">
+        <v>17</v>
+      </c>
       <c r="E7" s="12"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13" t="s">
         <v>18</v>
       </c>
@@ -1208,15 +1298,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17" t="s">
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1228,8 +1318,8 @@
       <c r="C11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="24" t="s">
+      <c r="D11" s="16"/>
+      <c r="E11" s="23" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1242,7 +1332,7 @@
         <v>43</v>
       </c>
       <c r="D12" s="15"/>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="16" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1255,7 +1345,7 @@
         <v>46</v>
       </c>
       <c r="D13" s="15"/>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="16" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1264,127 +1354,123 @@
         <f aca="false">B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="n">
         <f aca="false">B14+1</f>
         <v>6</v>
       </c>
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
-      <c r="E15" s="17"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E15" s="16"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
       </c>
       <c r="C16" s="15"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
       <c r="C17" s="15"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="n">
         <f aca="false">B17+1</f>
         <v>9</v>
       </c>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
-      <c r="E18" s="17"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E18" s="16"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="n">
         <f aca="false">B18+1</f>
         <v>10</v>
       </c>
       <c r="C19" s="15"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="n">
         <f aca="false">B19+1</f>
         <v>11</v>
       </c>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
-      <c r="E20" s="17"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E20" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="n">
         <f aca="false">B20+1</f>
         <v>12</v>
       </c>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
-      <c r="E21" s="17"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E21" s="16"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="n">
         <f aca="false">B21+1</f>
         <v>13</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
-      <c r="E22" s="17"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E22" s="16"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="n">
         <f aca="false">B22+1</f>
         <v>14</v>
       </c>
       <c r="C23" s="15"/>
       <c r="D23" s="15"/>
-      <c r="E23" s="17"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E23" s="16"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="n">
         <f aca="false">B23+1</f>
         <v>15</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
-      <c r="E24" s="17"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E24" s="16"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="n">
         <f aca="false">B24+1</f>
         <v>16</v>
       </c>
       <c r="C25" s="15"/>
       <c r="D25" s="15"/>
-      <c r="E25" s="17"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E25" s="16"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="n">
         <f aca="false">B25+1</f>
         <v>17</v>
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
-      <c r="E26" s="17"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="19" t="s">
+      <c r="E26" s="16"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C28" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="20"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="15" t="n">
         <v>0.5</v>
       </c>
@@ -1415,16 +1501,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.91015625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.45"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.72"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1438,9 +1524,9 @@
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1453,7 +1539,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
@@ -1464,14 +1550,14 @@
         <v>233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="25" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C4" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="26"/>
+      <c r="D4" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="25"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1482,14 +1568,14 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="25" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" s="27"/>
+      <c r="D5" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="26"/>
       <c r="H5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1500,7 +1586,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="10"/>
       <c r="C6" s="11" t="s">
         <v>15</v>
@@ -1508,14 +1594,16 @@
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="12" t="s">
+        <v>51</v>
+      </c>
       <c r="E7" s="12"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13" t="s">
         <v>18</v>
       </c>
@@ -1529,199 +1617,215 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="n">
         <f aca="false">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15"/>
+      <c r="C11" s="15" t="s">
+        <v>54</v>
+      </c>
       <c r="D11" s="15"/>
-      <c r="E11" s="17"/>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E11" s="16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="n">
         <f aca="false">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="15"/>
+      <c r="C12" s="15" t="s">
+        <v>52</v>
+      </c>
       <c r="D12" s="15"/>
-      <c r="E12" s="17"/>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E12" s="16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="n">
         <f aca="false">B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="n">
         <f aca="false">B13+1</f>
         <v>5</v>
       </c>
       <c r="C14" s="15"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="n">
         <f aca="false">B14+1</f>
         <v>6</v>
       </c>
       <c r="C15" s="15"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
       </c>
       <c r="C16" s="15"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
       <c r="C17" s="15"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="n">
         <f aca="false">B17+1</f>
         <v>9</v>
       </c>
       <c r="C18" s="15"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="n">
         <f aca="false">B18+1</f>
         <v>10</v>
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
-      <c r="E19" s="17"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E19" s="16"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="n">
         <f aca="false">B19+1</f>
         <v>11</v>
       </c>
       <c r="C20" s="15"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="n">
         <f aca="false">B20+1</f>
         <v>12</v>
       </c>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
-      <c r="E21" s="17"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E21" s="16"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="n">
         <f aca="false">B21+1</f>
         <v>13</v>
       </c>
       <c r="C22" s="15"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="n">
         <f aca="false">B22+1</f>
         <v>14</v>
       </c>
       <c r="C23" s="15"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="n">
         <f aca="false">B23+1</f>
         <v>15</v>
       </c>
       <c r="C24" s="15"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="n">
         <f aca="false">B24+1</f>
         <v>16</v>
       </c>
       <c r="C25" s="15"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="n">
         <f aca="false">B25+1</f>
         <v>17</v>
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
-      <c r="E26" s="17"/>
-    </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E26" s="16"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="n">
         <f aca="false">B26+1</f>
         <v>18</v>
       </c>
       <c r="C27" s="15"/>
-      <c r="D27" s="17"/>
+      <c r="D27" s="16"/>
       <c r="E27" s="15"/>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="n">
         <f aca="false">B27+1</f>
         <v>19</v>
       </c>
       <c r="C28" s="15"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="n">
         <f aca="false">B28+1</f>
         <v>20</v>
       </c>
       <c r="C29" s="15"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="n">
         <f aca="false">B29+1</f>
         <v>21</v>
       </c>
       <c r="C30" s="15"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="19" t="s">
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="20"/>
+      <c r="D32" s="19"/>
       <c r="E32" s="15"/>
     </row>
   </sheetData>
@@ -1750,17 +1854,17 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.91015625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.63"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.58"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.72"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,9 +1878,9 @@
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1789,7 +1893,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
@@ -1800,12 +1904,12 @@
         <v>233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C4" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1816,7 +1920,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="11" t="s">
         <v>15</v>
       </c>
@@ -1832,247 +1936,295 @@
         <v>233</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="10"/>
       <c r="C6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="12"/>
+      <c r="D6" s="12" t="s">
+        <v>51</v>
+      </c>
       <c r="E6" s="12"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="n">
+      <c r="C10" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="27" t="n">
         <f aca="false">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="n">
+      <c r="C11" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="27" t="n">
         <f aca="false">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="n">
+      <c r="C12" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="27" t="n">
         <f aca="false">B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="n">
+      <c r="C13" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" s="29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="27" t="n">
         <f aca="false">B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="n">
+      <c r="C14" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="F14" s="29" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="27" t="n">
         <f aca="false">B14+1</f>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="n">
+      <c r="C15" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="F15" s="29" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="27" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="n">
+      <c r="C16" s="28"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="27" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="n">
+      <c r="C17" s="28"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="27" t="n">
         <f aca="false">B17+1</f>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="n">
+      <c r="C18" s="28"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="27" t="n">
         <f aca="false">B18+1</f>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="n">
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="27" t="n">
         <f aca="false">B19+1</f>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="n">
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="27" t="n">
         <f aca="false">B20+1</f>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="n">
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="27" t="n">
         <f aca="false">B21+1</f>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="n">
+      <c r="C22" s="28"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="27" t="n">
         <f aca="false">B22+1</f>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="6" t="n">
+      <c r="C23" s="28"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="27" t="n">
         <f aca="false">B23+1</f>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="n">
+      <c r="C24" s="28"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="27" t="n">
         <f aca="false">B24+1</f>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="6" t="n">
+      <c r="C25" s="28"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="27" t="n">
         <f aca="false">B25+1</f>
         <v>17</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-    </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="n">
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="27" t="n">
         <f aca="false">B26+1</f>
         <v>18</v>
       </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="6" t="n">
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="27" t="n">
         <f aca="false">B27+1</f>
         <v>19</v>
       </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="6" t="n">
+      <c r="C28" s="28"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="27" t="n">
         <f aca="false">B28+1</f>
         <v>20</v>
       </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="6" t="n">
+      <c r="C29" s="28"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="27" t="n">
         <f aca="false">B29+1</f>
         <v>21</v>
       </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="29"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>